<commit_message>
Add Transcript History sheet to Template 8 for grade history
Adds a second sheet 'Transcript History' to Template 8 (Student Profiles)
for collecting historical final grades per student per course. Used by
the engine for two critical validations:
1. Duplicate request detection — flag courses already completed
2. Prerequisite validation — confirm required prior courses were passed

Columns: Student ID, Academic Year, Course Code, Course Title, Department,
Credits, Final Grade, Passed (Y/N), Grade Level When Taken, Notes

This is a required feature for the commercial product build.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_8_Student_Profiles.xlsx
+++ b/templates/Template_8_Student_Profiles.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Student Profiles" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transcript History" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,8 +69,36 @@
       <color rgb="00999999"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B4965"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="007A7A7A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00926B18"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B4965"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002D6A4F"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +141,12 @@
         <bgColor rgb="00EEF0F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -139,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -161,6 +196,11 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -60747,4 +60787,601 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>STUDENT TRANSCRIPT HISTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Used by the engine for: (1) Duplicate request detection — flag courses already completed  (2) Prerequisite validation — confirm required prior courses were passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Academic Year</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Course Code</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Course Title</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Credits</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Final Grade</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>Grade Level When Taken</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="n">
+        <v>106212</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Composition &amp; Literature</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" s="11" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="n">
+        <v>106212</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>410</v>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Algebra I</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="n">
+        <v>106212</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>810</v>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Theology 9</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Theology</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="n">
+        <v>106212</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>610</v>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Phys Ed/Health</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="n">
+        <v>106212</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>112</v>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Composition &amp; Literature</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="J9" s="11" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
+        <v>106212</v>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>510</v>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Earth Science</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="J10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
+        <v>115945</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>111</v>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Composition &amp; Literature H</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="J11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
+        <v>115945</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>411</v>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Geometry H</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="J12" s="11" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>HOW TO USE:</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Export transcript/grade history from your SIS. One row per student per completed course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Student ID:</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Must match the Student ID in the Student Profiles sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Academic Year:</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Format: "2025-26", "2024-25", etc. Include all available years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Final Grade:</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Letter grade (A+, A, A-, B+, B, B-, C+, C, C-, D, F) or numeric (95, 87, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Passed:</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>"Y" if credit was earned, "N" if failed/incomplete/withdrawn</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>PURPOSE 1:</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>DUPLICATE DETECTION — If a student requests course 410 but already passed it, the engine flags it as an error</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>PURPOSE 2:</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>PREREQUISITE CHECK — If course 430 requires 410, the engine verifies the student passed 410 before allowing 430</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>TYPICAL SIZE:</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>About 5,000-15,000 rows depending on how many years of history you include</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>MINIMUM:</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>At least the most recent completed year (2025-26) is needed. 2-3 years is ideal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>DELETE:</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Delete the yellow example rows before uploading — they are just format guides.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="B19:J19"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B22:J22"/>
+    <mergeCell ref="B17:J17"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B16:J16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Flag 40 LEO I students in Template 8
All 40 students requesting course 734 (LEO I) now have LEO I = Y
in T8. LEO I is SSP (+25 priority points). 8 of these students had
no Pathway or Academic Support flag and were receiving 0 SSP points.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_8_Student_Profiles.xlsx
+++ b/templates/Template_8_Student_Profiles.xlsx
@@ -2461,7 +2461,7 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H100" s="4" t="inlineStr">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H109" s="4" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H110" s="4" t="inlineStr">
@@ -7087,7 +7087,7 @@
       </c>
       <c r="G134" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H134" s="4" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="G148" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H148" s="4" t="inlineStr">
@@ -11905,7 +11905,7 @@
       </c>
       <c r="G232" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H232" s="4" t="inlineStr">
@@ -12542,7 +12542,7 @@
       </c>
       <c r="G245" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H245" s="4" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="G249" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H249" s="4" t="inlineStr">
@@ -12938,7 +12938,7 @@
       </c>
       <c r="G253" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H253" s="4" t="inlineStr">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="G266" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H266" s="4" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="G287" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr">
@@ -15000,7 +15000,7 @@
       </c>
       <c r="G295" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H295" s="4" t="inlineStr">
@@ -15951,7 +15951,7 @@
       </c>
       <c r="G314" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H314" s="4" t="inlineStr">
@@ -16147,7 +16147,7 @@
       </c>
       <c r="G318" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H318" s="4" t="inlineStr">
@@ -16841,7 +16841,7 @@
       </c>
       <c r="G332" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H332" s="4" t="inlineStr">
@@ -18556,7 +18556,7 @@
       </c>
       <c r="G367" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H367" s="4" t="inlineStr">
@@ -18850,7 +18850,7 @@
       </c>
       <c r="G373" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H373" s="4" t="inlineStr">
@@ -19344,7 +19344,7 @@
       </c>
       <c r="G383" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H383" s="4" t="inlineStr">
@@ -19593,7 +19593,7 @@
       </c>
       <c r="G388" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H388" s="4" t="inlineStr">
@@ -19838,7 +19838,7 @@
       </c>
       <c r="G393" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H393" s="4" t="inlineStr">
@@ -21112,7 +21112,7 @@
       </c>
       <c r="G419" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H419" s="4" t="inlineStr">
@@ -22635,7 +22635,7 @@
       </c>
       <c r="G450" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H450" s="4" t="inlineStr">
@@ -23325,7 +23325,7 @@
       </c>
       <c r="G464" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H464" s="4" t="inlineStr">
@@ -24799,7 +24799,7 @@
       </c>
       <c r="G494" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H494" s="4" t="inlineStr">
@@ -25195,7 +25195,7 @@
       </c>
       <c r="G502" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H502" s="4" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="G522" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H522" s="4" t="inlineStr">
@@ -27122,7 +27122,7 @@
       </c>
       <c r="G541" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H541" s="4" t="inlineStr">
@@ -28690,7 +28690,7 @@
       </c>
       <c r="G573" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H573" s="4" t="inlineStr">
@@ -30017,7 +30017,7 @@
       </c>
       <c r="G600" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H600" s="4" t="inlineStr">
@@ -30066,7 +30066,7 @@
       </c>
       <c r="G601" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H601" s="4" t="inlineStr">
@@ -30605,7 +30605,7 @@
       </c>
       <c r="G612" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H612" s="4" t="inlineStr">
@@ -33790,7 +33790,7 @@
       </c>
       <c r="G677" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H677" s="4" t="inlineStr">
@@ -35260,7 +35260,7 @@
       </c>
       <c r="G707" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H707" s="4" t="inlineStr">
@@ -36534,7 +36534,7 @@
       </c>
       <c r="G733" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H733" s="4" t="inlineStr">
@@ -38008,7 +38008,7 @@
       </c>
       <c r="G763" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H763" s="4" t="inlineStr">
@@ -38453,7 +38453,7 @@
       </c>
       <c r="G772" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H772" s="4" t="inlineStr">
@@ -38845,7 +38845,7 @@
       </c>
       <c r="G780" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H780" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Fix #10: Remove duplicate student 116597 (Giordano, Joseph) from T8
- Deleted exact duplicate row 660 (identical to row 659)
- Student retained once with correct data (Gr9, Business pathway)
- T8 Sheet 1 now 804 unique students, 0 duplicates

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_8_Student_Profiles.xlsx
+++ b/templates/Template_8_Student_Profiles.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K807"/>
+  <dimension ref="A1:K806"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" style="6" min="1" max="1"/>
@@ -33057,20 +33057,20 @@
     </row>
     <row r="660">
       <c r="A660" s="8" t="n">
-        <v>116597</v>
+        <v>116602</v>
       </c>
       <c r="B660" s="8" t="inlineStr">
         <is>
-          <t>Giordano</t>
+          <t>Singh</t>
         </is>
       </c>
       <c r="C660" s="8" t="inlineStr">
         <is>
-          <t>Joseph</t>
+          <t>Harjeevan</t>
         </is>
       </c>
       <c r="D660" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E660" s="8" t="inlineStr">
         <is>
@@ -33094,7 +33094,7 @@
       </c>
       <c r="I660" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J660" s="8" t="n"/>
@@ -33106,16 +33106,16 @@
     </row>
     <row r="661">
       <c r="A661" s="8" t="n">
-        <v>116602</v>
+        <v>116607</v>
       </c>
       <c r="B661" s="8" t="inlineStr">
         <is>
-          <t>Singh</t>
+          <t>Webster</t>
         </is>
       </c>
       <c r="C661" s="8" t="inlineStr">
         <is>
-          <t>Harjeevan</t>
+          <t>Andrew</t>
         </is>
       </c>
       <c r="D661" s="8" t="n">
@@ -33143,7 +33143,7 @@
       </c>
       <c r="I661" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J661" s="8" t="n"/>
@@ -33155,20 +33155,20 @@
     </row>
     <row r="662">
       <c r="A662" s="8" t="n">
-        <v>116607</v>
+        <v>116614</v>
       </c>
       <c r="B662" s="8" t="inlineStr">
         <is>
-          <t>Webster</t>
+          <t>Fernandez</t>
         </is>
       </c>
       <c r="C662" s="8" t="inlineStr">
         <is>
-          <t>Andrew</t>
+          <t>Jayden</t>
         </is>
       </c>
       <c r="D662" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E662" s="8" t="inlineStr">
         <is>
@@ -33192,7 +33192,7 @@
       </c>
       <c r="I662" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="J662" s="8" t="n"/>
@@ -33204,16 +33204,16 @@
     </row>
     <row r="663">
       <c r="A663" s="8" t="n">
-        <v>116614</v>
+        <v>116616</v>
       </c>
       <c r="B663" s="8" t="inlineStr">
         <is>
-          <t>Fernandez</t>
+          <t>Sernack</t>
         </is>
       </c>
       <c r="C663" s="8" t="inlineStr">
         <is>
-          <t>Jayden</t>
+          <t>Imran</t>
         </is>
       </c>
       <c r="D663" s="8" t="n">
@@ -33241,7 +33241,7 @@
       </c>
       <c r="I663" s="8" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J663" s="8" t="n"/>
@@ -33253,16 +33253,16 @@
     </row>
     <row r="664">
       <c r="A664" s="8" t="n">
-        <v>116616</v>
+        <v>116624</v>
       </c>
       <c r="B664" s="8" t="inlineStr">
         <is>
-          <t>Sernack</t>
+          <t>Cho</t>
         </is>
       </c>
       <c r="C664" s="8" t="inlineStr">
         <is>
-          <t>Imran</t>
+          <t>Adrian</t>
         </is>
       </c>
       <c r="D664" s="8" t="n">
@@ -33290,7 +33290,7 @@
       </c>
       <c r="I664" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J664" s="8" t="n"/>
@@ -33302,20 +33302,20 @@
     </row>
     <row r="665">
       <c r="A665" s="8" t="n">
-        <v>116624</v>
+        <v>116628</v>
       </c>
       <c r="B665" s="8" t="inlineStr">
         <is>
-          <t>Cho</t>
+          <t>McConnell</t>
         </is>
       </c>
       <c r="C665" s="8" t="inlineStr">
         <is>
-          <t>Adrian</t>
+          <t>Lincoln</t>
         </is>
       </c>
       <c r="D665" s="8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E665" s="8" t="inlineStr">
         <is>
@@ -33339,7 +33339,7 @@
       </c>
       <c r="I665" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J665" s="8" t="n"/>
@@ -33351,20 +33351,20 @@
     </row>
     <row r="666">
       <c r="A666" s="8" t="n">
-        <v>116628</v>
+        <v>116729</v>
       </c>
       <c r="B666" s="8" t="inlineStr">
         <is>
-          <t>McConnell</t>
+          <t>Bouab</t>
         </is>
       </c>
       <c r="C666" s="8" t="inlineStr">
         <is>
-          <t>Lincoln</t>
+          <t>Acelan</t>
         </is>
       </c>
       <c r="D666" s="8" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E666" s="8" t="inlineStr">
         <is>
@@ -33388,7 +33388,7 @@
       </c>
       <c r="I666" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Fine Arts</t>
         </is>
       </c>
       <c r="J666" s="8" t="n"/>
@@ -33400,16 +33400,16 @@
     </row>
     <row r="667">
       <c r="A667" s="8" t="n">
-        <v>116729</v>
+        <v>116807</v>
       </c>
       <c r="B667" s="8" t="inlineStr">
         <is>
-          <t>Bouab</t>
+          <t>Antigua</t>
         </is>
       </c>
       <c r="C667" s="8" t="inlineStr">
         <is>
-          <t>Acelan</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="D667" s="8" t="n">
@@ -33437,7 +33437,7 @@
       </c>
       <c r="I667" s="8" t="inlineStr">
         <is>
-          <t>Fine Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J667" s="8" t="n"/>
@@ -33449,20 +33449,20 @@
     </row>
     <row r="668">
       <c r="A668" s="8" t="n">
-        <v>116807</v>
+        <v>116815</v>
       </c>
       <c r="B668" s="8" t="inlineStr">
         <is>
-          <t>Antigua</t>
+          <t>DellaVolpe</t>
         </is>
       </c>
       <c r="C668" s="8" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Louis</t>
         </is>
       </c>
       <c r="D668" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E668" s="8" t="inlineStr">
         <is>
@@ -33481,12 +33481,12 @@
       </c>
       <c r="H668" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I668" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J668" s="8" t="n"/>
@@ -33498,20 +33498,20 @@
     </row>
     <row r="669">
       <c r="A669" s="8" t="n">
-        <v>116815</v>
+        <v>116837</v>
       </c>
       <c r="B669" s="8" t="inlineStr">
         <is>
-          <t>DellaVolpe</t>
+          <t>Petrino</t>
         </is>
       </c>
       <c r="C669" s="8" t="inlineStr">
         <is>
-          <t>Louis</t>
+          <t>Jake</t>
         </is>
       </c>
       <c r="D669" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E669" s="8" t="inlineStr">
         <is>
@@ -33530,12 +33530,12 @@
       </c>
       <c r="H669" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I669" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J669" s="8" t="n"/>
@@ -33547,16 +33547,16 @@
     </row>
     <row r="670">
       <c r="A670" s="8" t="n">
-        <v>116837</v>
+        <v>116861</v>
       </c>
       <c r="B670" s="8" t="inlineStr">
         <is>
-          <t>Petrino</t>
+          <t>Uhl</t>
         </is>
       </c>
       <c r="C670" s="8" t="inlineStr">
         <is>
-          <t>Jake</t>
+          <t>Liam</t>
         </is>
       </c>
       <c r="D670" s="8" t="n">
@@ -33584,7 +33584,7 @@
       </c>
       <c r="I670" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J670" s="8" t="n"/>
@@ -33596,20 +33596,20 @@
     </row>
     <row r="671">
       <c r="A671" s="8" t="n">
-        <v>116861</v>
+        <v>116892</v>
       </c>
       <c r="B671" s="8" t="inlineStr">
         <is>
-          <t>Uhl</t>
+          <t>Boggis</t>
         </is>
       </c>
       <c r="C671" s="8" t="inlineStr">
         <is>
-          <t>Liam</t>
+          <t>Dean</t>
         </is>
       </c>
       <c r="D671" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E671" s="8" t="inlineStr">
         <is>
@@ -33633,7 +33633,7 @@
       </c>
       <c r="I671" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J671" s="8" t="n"/>
@@ -33645,20 +33645,20 @@
     </row>
     <row r="672">
       <c r="A672" s="8" t="n">
-        <v>116892</v>
+        <v>116919</v>
       </c>
       <c r="B672" s="8" t="inlineStr">
         <is>
-          <t>Boggis</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="C672" s="8" t="inlineStr">
         <is>
-          <t>Dean</t>
+          <t>Marco</t>
         </is>
       </c>
       <c r="D672" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E672" s="8" t="inlineStr">
         <is>
@@ -33682,7 +33682,7 @@
       </c>
       <c r="I672" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J672" s="8" t="n"/>
@@ -33694,16 +33694,16 @@
     </row>
     <row r="673">
       <c r="A673" s="8" t="n">
-        <v>116919</v>
+        <v>116924</v>
       </c>
       <c r="B673" s="8" t="inlineStr">
         <is>
-          <t>Domino</t>
+          <t>Sosa</t>
         </is>
       </c>
       <c r="C673" s="8" t="inlineStr">
         <is>
-          <t>Marco</t>
+          <t>Aiden</t>
         </is>
       </c>
       <c r="D673" s="8" t="n">
@@ -33743,20 +33743,20 @@
     </row>
     <row r="674">
       <c r="A674" s="8" t="n">
-        <v>116924</v>
+        <v>116930</v>
       </c>
       <c r="B674" s="8" t="inlineStr">
         <is>
-          <t>Sosa</t>
+          <t>Jean</t>
         </is>
       </c>
       <c r="C674" s="8" t="inlineStr">
         <is>
-          <t>Aiden</t>
+          <t>Jackson-Lucas</t>
         </is>
       </c>
       <c r="D674" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E674" s="8" t="inlineStr">
         <is>
@@ -33780,7 +33780,7 @@
       </c>
       <c r="I674" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Communication Arts</t>
         </is>
       </c>
       <c r="J674" s="8" t="n"/>
@@ -33792,20 +33792,20 @@
     </row>
     <row r="675">
       <c r="A675" s="8" t="n">
-        <v>116930</v>
+        <v>116969</v>
       </c>
       <c r="B675" s="8" t="inlineStr">
         <is>
-          <t>Jean</t>
+          <t>Mack</t>
         </is>
       </c>
       <c r="C675" s="8" t="inlineStr">
         <is>
-          <t>Jackson-Lucas</t>
+          <t>Zah’kyai</t>
         </is>
       </c>
       <c r="D675" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E675" s="8" t="inlineStr">
         <is>
@@ -33829,7 +33829,7 @@
       </c>
       <c r="I675" s="8" t="inlineStr">
         <is>
-          <t>Communication Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J675" s="8" t="n"/>
@@ -33841,20 +33841,20 @@
     </row>
     <row r="676">
       <c r="A676" s="8" t="n">
-        <v>116969</v>
+        <v>116980</v>
       </c>
       <c r="B676" s="8" t="inlineStr">
         <is>
-          <t>Mack</t>
+          <t>Adin</t>
         </is>
       </c>
       <c r="C676" s="8" t="inlineStr">
         <is>
-          <t>Zah’kyai</t>
+          <t>Logan</t>
         </is>
       </c>
       <c r="D676" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E676" s="8" t="inlineStr">
         <is>
@@ -33878,7 +33878,7 @@
       </c>
       <c r="I676" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="J676" s="8" t="n"/>
@@ -33890,20 +33890,20 @@
     </row>
     <row r="677">
       <c r="A677" s="8" t="n">
-        <v>116980</v>
+        <v>116994</v>
       </c>
       <c r="B677" s="8" t="inlineStr">
         <is>
-          <t>Adin</t>
+          <t>Moore</t>
         </is>
       </c>
       <c r="C677" s="8" t="inlineStr">
         <is>
-          <t>Logan</t>
+          <t>Isaac</t>
         </is>
       </c>
       <c r="D677" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E677" s="8" t="inlineStr">
         <is>
@@ -33927,7 +33927,7 @@
       </c>
       <c r="I677" s="8" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J677" s="8" t="n"/>
@@ -33939,16 +33939,16 @@
     </row>
     <row r="678">
       <c r="A678" s="8" t="n">
-        <v>116994</v>
+        <v>117092</v>
       </c>
       <c r="B678" s="8" t="inlineStr">
         <is>
-          <t>Moore</t>
+          <t>Fabiano</t>
         </is>
       </c>
       <c r="C678" s="8" t="inlineStr">
         <is>
-          <t>Isaac</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="D678" s="8" t="n">
@@ -33988,16 +33988,16 @@
     </row>
     <row r="679">
       <c r="A679" s="8" t="n">
-        <v>117092</v>
+        <v>117097</v>
       </c>
       <c r="B679" s="8" t="inlineStr">
         <is>
-          <t>Fabiano</t>
+          <t>Gallucci</t>
         </is>
       </c>
       <c r="C679" s="8" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="D679" s="8" t="n">
@@ -34037,20 +34037,20 @@
     </row>
     <row r="680">
       <c r="A680" s="8" t="n">
-        <v>117097</v>
+        <v>117105</v>
       </c>
       <c r="B680" s="8" t="inlineStr">
         <is>
-          <t>Gallucci</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="C680" s="8" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Ca'Si</t>
         </is>
       </c>
       <c r="D680" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E680" s="8" t="inlineStr">
         <is>
@@ -34074,7 +34074,7 @@
       </c>
       <c r="I680" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J680" s="8" t="n"/>
@@ -34086,20 +34086,20 @@
     </row>
     <row r="681">
       <c r="A681" s="8" t="n">
-        <v>117105</v>
+        <v>117132</v>
       </c>
       <c r="B681" s="8" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Jean-Marie</t>
         </is>
       </c>
       <c r="C681" s="8" t="inlineStr">
         <is>
-          <t>Ca'Si</t>
+          <t>Samuel</t>
         </is>
       </c>
       <c r="D681" s="8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E681" s="8" t="inlineStr">
         <is>
@@ -34135,20 +34135,20 @@
     </row>
     <row r="682">
       <c r="A682" s="8" t="n">
-        <v>117132</v>
+        <v>117136</v>
       </c>
       <c r="B682" s="8" t="inlineStr">
         <is>
-          <t>Jean-Marie</t>
+          <t>Park</t>
         </is>
       </c>
       <c r="C682" s="8" t="inlineStr">
         <is>
-          <t>Samuel</t>
+          <t>Aiden</t>
         </is>
       </c>
       <c r="D682" s="8" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E682" s="8" t="inlineStr">
         <is>
@@ -34172,7 +34172,7 @@
       </c>
       <c r="I682" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J682" s="8" t="n"/>
@@ -34184,20 +34184,20 @@
     </row>
     <row r="683">
       <c r="A683" s="8" t="n">
-        <v>117136</v>
+        <v>117153</v>
       </c>
       <c r="B683" s="8" t="inlineStr">
         <is>
-          <t>Park</t>
+          <t>Brown</t>
         </is>
       </c>
       <c r="C683" s="8" t="inlineStr">
         <is>
-          <t>Aiden</t>
+          <t>Marcus</t>
         </is>
       </c>
       <c r="D683" s="8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E683" s="8" t="inlineStr">
         <is>
@@ -34221,7 +34221,7 @@
       </c>
       <c r="I683" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J683" s="8" t="n"/>
@@ -34233,20 +34233,20 @@
     </row>
     <row r="684">
       <c r="A684" s="8" t="n">
-        <v>117153</v>
+        <v>117239</v>
       </c>
       <c r="B684" s="8" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>Tristani</t>
         </is>
       </c>
       <c r="C684" s="8" t="inlineStr">
         <is>
-          <t>Marcus</t>
+          <t>Antonio</t>
         </is>
       </c>
       <c r="D684" s="8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E684" s="8" t="inlineStr">
         <is>
@@ -34282,16 +34282,16 @@
     </row>
     <row r="685">
       <c r="A685" s="8" t="n">
-        <v>117239</v>
+        <v>117247</v>
       </c>
       <c r="B685" s="8" t="inlineStr">
         <is>
-          <t>Tristani</t>
+          <t>Ohnegian</t>
         </is>
       </c>
       <c r="C685" s="8" t="inlineStr">
         <is>
-          <t>Antonio</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="D685" s="8" t="n">
@@ -34331,20 +34331,20 @@
     </row>
     <row r="686">
       <c r="A686" s="8" t="n">
-        <v>117247</v>
+        <v>117259</v>
       </c>
       <c r="B686" s="8" t="inlineStr">
         <is>
-          <t>Ohnegian</t>
+          <t>Bredy</t>
         </is>
       </c>
       <c r="C686" s="8" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Malachi</t>
         </is>
       </c>
       <c r="D686" s="8" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E686" s="8" t="inlineStr">
         <is>
@@ -34368,7 +34368,7 @@
       </c>
       <c r="I686" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Communication Arts</t>
         </is>
       </c>
       <c r="J686" s="8" t="n"/>
@@ -34380,16 +34380,16 @@
     </row>
     <row r="687">
       <c r="A687" s="8" t="n">
-        <v>117259</v>
+        <v>117274</v>
       </c>
       <c r="B687" s="8" t="inlineStr">
         <is>
-          <t>Bredy</t>
+          <t>Casillo</t>
         </is>
       </c>
       <c r="C687" s="8" t="inlineStr">
         <is>
-          <t>Malachi</t>
+          <t>Joseph</t>
         </is>
       </c>
       <c r="D687" s="8" t="n">
@@ -34417,7 +34417,7 @@
       </c>
       <c r="I687" s="8" t="inlineStr">
         <is>
-          <t>Communication Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J687" s="8" t="n"/>
@@ -34429,16 +34429,16 @@
     </row>
     <row r="688">
       <c r="A688" s="8" t="n">
-        <v>117274</v>
+        <v>117280</v>
       </c>
       <c r="B688" s="8" t="inlineStr">
         <is>
-          <t>Casillo</t>
+          <t>Solow</t>
         </is>
       </c>
       <c r="C688" s="8" t="inlineStr">
         <is>
-          <t>Joseph</t>
+          <t>Jacob</t>
         </is>
       </c>
       <c r="D688" s="8" t="n">
@@ -34466,7 +34466,7 @@
       </c>
       <c r="I688" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Communication Arts</t>
         </is>
       </c>
       <c r="J688" s="8" t="n"/>
@@ -34478,16 +34478,16 @@
     </row>
     <row r="689">
       <c r="A689" s="8" t="n">
-        <v>117280</v>
+        <v>117333</v>
       </c>
       <c r="B689" s="8" t="inlineStr">
         <is>
-          <t>Solow</t>
+          <t>Setoodeh</t>
         </is>
       </c>
       <c r="C689" s="8" t="inlineStr">
         <is>
-          <t>Jacob</t>
+          <t>Devon</t>
         </is>
       </c>
       <c r="D689" s="8" t="n">
@@ -34515,7 +34515,7 @@
       </c>
       <c r="I689" s="8" t="inlineStr">
         <is>
-          <t>Communication Arts</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J689" s="8" t="n"/>
@@ -34527,16 +34527,16 @@
     </row>
     <row r="690">
       <c r="A690" s="8" t="n">
-        <v>117333</v>
+        <v>117344</v>
       </c>
       <c r="B690" s="8" t="inlineStr">
         <is>
-          <t>Setoodeh</t>
+          <t>Christian</t>
         </is>
       </c>
       <c r="C690" s="8" t="inlineStr">
         <is>
-          <t>Devon</t>
+          <t>Xavier</t>
         </is>
       </c>
       <c r="D690" s="8" t="n">
@@ -34576,16 +34576,16 @@
     </row>
     <row r="691">
       <c r="A691" s="8" t="n">
-        <v>117344</v>
+        <v>117347</v>
       </c>
       <c r="B691" s="8" t="inlineStr">
         <is>
-          <t>Christian</t>
+          <t>Pacilio</t>
         </is>
       </c>
       <c r="C691" s="8" t="inlineStr">
         <is>
-          <t>Xavier</t>
+          <t>Neil</t>
         </is>
       </c>
       <c r="D691" s="8" t="n">
@@ -34613,7 +34613,7 @@
       </c>
       <c r="I691" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J691" s="8" t="n"/>
@@ -34625,16 +34625,16 @@
     </row>
     <row r="692">
       <c r="A692" s="8" t="n">
-        <v>117347</v>
+        <v>117354</v>
       </c>
       <c r="B692" s="8" t="inlineStr">
         <is>
-          <t>Pacilio</t>
+          <t>Kennedy</t>
         </is>
       </c>
       <c r="C692" s="8" t="inlineStr">
         <is>
-          <t>Neil</t>
+          <t>Grant</t>
         </is>
       </c>
       <c r="D692" s="8" t="n">
@@ -34674,20 +34674,20 @@
     </row>
     <row r="693">
       <c r="A693" s="8" t="n">
-        <v>117354</v>
+        <v>117392</v>
       </c>
       <c r="B693" s="8" t="inlineStr">
         <is>
-          <t>Kennedy</t>
+          <t>Actisdano</t>
         </is>
       </c>
       <c r="C693" s="8" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="D693" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E693" s="8" t="inlineStr">
         <is>
@@ -34711,7 +34711,7 @@
       </c>
       <c r="I693" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J693" s="8" t="n"/>
@@ -34723,20 +34723,20 @@
     </row>
     <row r="694">
       <c r="A694" s="8" t="n">
-        <v>117392</v>
+        <v>117398</v>
       </c>
       <c r="B694" s="8" t="inlineStr">
         <is>
-          <t>Actisdano</t>
+          <t>Perkell</t>
         </is>
       </c>
       <c r="C694" s="8" t="inlineStr">
         <is>
-          <t>Nicholas</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="D694" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E694" s="8" t="inlineStr">
         <is>
@@ -34760,7 +34760,7 @@
       </c>
       <c r="I694" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J694" s="8" t="n"/>
@@ -34772,16 +34772,16 @@
     </row>
     <row r="695">
       <c r="A695" s="8" t="n">
-        <v>117398</v>
+        <v>117409</v>
       </c>
       <c r="B695" s="8" t="inlineStr">
         <is>
-          <t>Perkell</t>
+          <t>Philp</t>
         </is>
       </c>
       <c r="C695" s="8" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Mason</t>
         </is>
       </c>
       <c r="D695" s="8" t="n">
@@ -34821,20 +34821,20 @@
     </row>
     <row r="696">
       <c r="A696" s="8" t="n">
-        <v>117409</v>
+        <v>117427</v>
       </c>
       <c r="B696" s="8" t="inlineStr">
         <is>
-          <t>Philp</t>
+          <t>Irving</t>
         </is>
       </c>
       <c r="C696" s="8" t="inlineStr">
         <is>
-          <t>Mason</t>
+          <t>Corey</t>
         </is>
       </c>
       <c r="D696" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E696" s="8" t="inlineStr">
         <is>
@@ -34858,7 +34858,7 @@
       </c>
       <c r="I696" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J696" s="8" t="n"/>
@@ -34870,20 +34870,20 @@
     </row>
     <row r="697">
       <c r="A697" s="8" t="n">
-        <v>117427</v>
+        <v>117436</v>
       </c>
       <c r="B697" s="8" t="inlineStr">
         <is>
-          <t>Irving</t>
+          <t>Laracy</t>
         </is>
       </c>
       <c r="C697" s="8" t="inlineStr">
         <is>
-          <t>Corey</t>
+          <t>Gregory</t>
         </is>
       </c>
       <c r="D697" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E697" s="8" t="inlineStr">
         <is>
@@ -34907,7 +34907,7 @@
       </c>
       <c r="I697" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J697" s="8" t="n"/>
@@ -34919,16 +34919,16 @@
     </row>
     <row r="698">
       <c r="A698" s="8" t="n">
-        <v>117436</v>
+        <v>117446</v>
       </c>
       <c r="B698" s="8" t="inlineStr">
         <is>
-          <t>Laracy</t>
+          <t>Leon-Ahuacatitan</t>
         </is>
       </c>
       <c r="C698" s="8" t="inlineStr">
         <is>
-          <t>Gregory</t>
+          <t>Gael</t>
         </is>
       </c>
       <c r="D698" s="8" t="n">
@@ -34956,7 +34956,7 @@
       </c>
       <c r="I698" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J698" s="8" t="n"/>
@@ -34968,16 +34968,16 @@
     </row>
     <row r="699">
       <c r="A699" s="8" t="n">
-        <v>117446</v>
+        <v>117452</v>
       </c>
       <c r="B699" s="8" t="inlineStr">
         <is>
-          <t>Leon-Ahuacatitan</t>
+          <t>McCormack</t>
         </is>
       </c>
       <c r="C699" s="8" t="inlineStr">
         <is>
-          <t>Gael</t>
+          <t>Rylan</t>
         </is>
       </c>
       <c r="D699" s="8" t="n">
@@ -35017,16 +35017,16 @@
     </row>
     <row r="700">
       <c r="A700" s="8" t="n">
-        <v>117452</v>
+        <v>117481</v>
       </c>
       <c r="B700" s="8" t="inlineStr">
         <is>
-          <t>McCormack</t>
+          <t>Dettlaff</t>
         </is>
       </c>
       <c r="C700" s="8" t="inlineStr">
         <is>
-          <t>Rylan</t>
+          <t>Donato</t>
         </is>
       </c>
       <c r="D700" s="8" t="n">
@@ -35054,7 +35054,7 @@
       </c>
       <c r="I700" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J700" s="8" t="n"/>
@@ -35066,20 +35066,20 @@
     </row>
     <row r="701">
       <c r="A701" s="8" t="n">
-        <v>117481</v>
+        <v>117590</v>
       </c>
       <c r="B701" s="8" t="inlineStr">
         <is>
-          <t>Dettlaff</t>
+          <t>Naudy</t>
         </is>
       </c>
       <c r="C701" s="8" t="inlineStr">
         <is>
-          <t>Donato</t>
+          <t>Enrique</t>
         </is>
       </c>
       <c r="D701" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E701" s="8" t="inlineStr">
         <is>
@@ -35103,7 +35103,7 @@
       </c>
       <c r="I701" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Fine Arts</t>
         </is>
       </c>
       <c r="J701" s="8" t="n"/>
@@ -35115,16 +35115,16 @@
     </row>
     <row r="702">
       <c r="A702" s="8" t="n">
-        <v>117590</v>
+        <v>117612</v>
       </c>
       <c r="B702" s="8" t="inlineStr">
         <is>
-          <t>Naudy</t>
+          <t>Dorsainville</t>
         </is>
       </c>
       <c r="C702" s="8" t="inlineStr">
         <is>
-          <t>Enrique</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="D702" s="8" t="n">
@@ -35152,7 +35152,7 @@
       </c>
       <c r="I702" s="8" t="inlineStr">
         <is>
-          <t>Fine Arts</t>
+          <t>Communication Arts</t>
         </is>
       </c>
       <c r="J702" s="8" t="n"/>
@@ -35164,20 +35164,20 @@
     </row>
     <row r="703">
       <c r="A703" s="8" t="n">
-        <v>117612</v>
+        <v>117628</v>
       </c>
       <c r="B703" s="8" t="inlineStr">
         <is>
-          <t>Dorsainville</t>
+          <t>De los Santos</t>
         </is>
       </c>
       <c r="C703" s="8" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Rodrigo</t>
         </is>
       </c>
       <c r="D703" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E703" s="8" t="inlineStr">
         <is>
@@ -35201,7 +35201,7 @@
       </c>
       <c r="I703" s="8" t="inlineStr">
         <is>
-          <t>Communication Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J703" s="8" t="n"/>
@@ -35213,16 +35213,16 @@
     </row>
     <row r="704">
       <c r="A704" s="8" t="n">
-        <v>117628</v>
+        <v>117653</v>
       </c>
       <c r="B704" s="8" t="inlineStr">
         <is>
-          <t>De los Santos</t>
+          <t>Jean Baptiste</t>
         </is>
       </c>
       <c r="C704" s="8" t="inlineStr">
         <is>
-          <t>Rodrigo</t>
+          <t>Miles</t>
         </is>
       </c>
       <c r="D704" s="8" t="n">
@@ -35250,7 +35250,7 @@
       </c>
       <c r="I704" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J704" s="8" t="n"/>
@@ -35262,20 +35262,20 @@
     </row>
     <row r="705">
       <c r="A705" s="8" t="n">
-        <v>117653</v>
+        <v>117698</v>
       </c>
       <c r="B705" s="8" t="inlineStr">
         <is>
-          <t>Jean Baptiste</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="C705" s="8" t="inlineStr">
         <is>
-          <t>Miles</t>
+          <t>Jamel</t>
         </is>
       </c>
       <c r="D705" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E705" s="8" t="inlineStr">
         <is>
@@ -35299,7 +35299,7 @@
       </c>
       <c r="I705" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>Communication Arts</t>
         </is>
       </c>
       <c r="J705" s="8" t="n"/>
@@ -35311,20 +35311,20 @@
     </row>
     <row r="706">
       <c r="A706" s="8" t="n">
-        <v>117698</v>
+        <v>117733</v>
       </c>
       <c r="B706" s="8" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Mistretta</t>
         </is>
       </c>
       <c r="C706" s="8" t="inlineStr">
         <is>
-          <t>Jamel</t>
+          <t>Joseph</t>
         </is>
       </c>
       <c r="D706" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E706" s="8" t="inlineStr">
         <is>
@@ -35348,7 +35348,7 @@
       </c>
       <c r="I706" s="8" t="inlineStr">
         <is>
-          <t>Communication Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J706" s="8" t="n"/>
@@ -35360,16 +35360,16 @@
     </row>
     <row r="707">
       <c r="A707" s="8" t="n">
-        <v>117733</v>
+        <v>117743</v>
       </c>
       <c r="B707" s="8" t="inlineStr">
         <is>
-          <t>Mistretta</t>
+          <t>Cruz</t>
         </is>
       </c>
       <c r="C707" s="8" t="inlineStr">
         <is>
-          <t>Joseph</t>
+          <t>Dante</t>
         </is>
       </c>
       <c r="D707" s="8" t="n">
@@ -35397,7 +35397,7 @@
       </c>
       <c r="I707" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="J707" s="8" t="n"/>
@@ -35409,16 +35409,16 @@
     </row>
     <row r="708">
       <c r="A708" s="8" t="n">
-        <v>117743</v>
+        <v>117752</v>
       </c>
       <c r="B708" s="8" t="inlineStr">
         <is>
-          <t>Cruz</t>
+          <t>Sabnani</t>
         </is>
       </c>
       <c r="C708" s="8" t="inlineStr">
         <is>
-          <t>Dante</t>
+          <t>Avish</t>
         </is>
       </c>
       <c r="D708" s="8" t="n">
@@ -35446,7 +35446,7 @@
       </c>
       <c r="I708" s="8" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J708" s="8" t="n"/>
@@ -35458,16 +35458,16 @@
     </row>
     <row r="709">
       <c r="A709" s="8" t="n">
-        <v>117752</v>
+        <v>117844</v>
       </c>
       <c r="B709" s="8" t="inlineStr">
         <is>
-          <t>Sabnani</t>
+          <t>Mims</t>
         </is>
       </c>
       <c r="C709" s="8" t="inlineStr">
         <is>
-          <t>Avish</t>
+          <t>Chayse</t>
         </is>
       </c>
       <c r="D709" s="8" t="n">
@@ -35507,16 +35507,16 @@
     </row>
     <row r="710">
       <c r="A710" s="8" t="n">
-        <v>117844</v>
+        <v>117848</v>
       </c>
       <c r="B710" s="8" t="inlineStr">
         <is>
-          <t>Mims</t>
+          <t>Zuena</t>
         </is>
       </c>
       <c r="C710" s="8" t="inlineStr">
         <is>
-          <t>Chayse</t>
+          <t>Philip</t>
         </is>
       </c>
       <c r="D710" s="8" t="n">
@@ -35556,16 +35556,16 @@
     </row>
     <row r="711">
       <c r="A711" s="8" t="n">
-        <v>117848</v>
+        <v>117857</v>
       </c>
       <c r="B711" s="8" t="inlineStr">
         <is>
-          <t>Zuena</t>
+          <t>Saume</t>
         </is>
       </c>
       <c r="C711" s="8" t="inlineStr">
         <is>
-          <t>Philip</t>
+          <t>David</t>
         </is>
       </c>
       <c r="D711" s="8" t="n">
@@ -35605,16 +35605,16 @@
     </row>
     <row r="712">
       <c r="A712" s="8" t="n">
-        <v>117857</v>
+        <v>117888</v>
       </c>
       <c r="B712" s="8" t="inlineStr">
         <is>
-          <t>Saume</t>
+          <t>Augustyn</t>
         </is>
       </c>
       <c r="C712" s="8" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Owen</t>
         </is>
       </c>
       <c r="D712" s="8" t="n">
@@ -35654,16 +35654,16 @@
     </row>
     <row r="713">
       <c r="A713" s="8" t="n">
-        <v>117888</v>
+        <v>117901</v>
       </c>
       <c r="B713" s="8" t="inlineStr">
         <is>
-          <t>Augustyn</t>
+          <t>Pinto</t>
         </is>
       </c>
       <c r="C713" s="8" t="inlineStr">
         <is>
-          <t>Owen</t>
+          <t>Niko</t>
         </is>
       </c>
       <c r="D713" s="8" t="n">
@@ -35703,16 +35703,16 @@
     </row>
     <row r="714">
       <c r="A714" s="8" t="n">
-        <v>117901</v>
+        <v>117907</v>
       </c>
       <c r="B714" s="8" t="inlineStr">
         <is>
-          <t>Pinto</t>
+          <t>Dimaras</t>
         </is>
       </c>
       <c r="C714" s="8" t="inlineStr">
         <is>
-          <t>Niko</t>
+          <t>Konstantinos</t>
         </is>
       </c>
       <c r="D714" s="8" t="n">
@@ -35752,16 +35752,16 @@
     </row>
     <row r="715">
       <c r="A715" s="8" t="n">
-        <v>117907</v>
+        <v>117941</v>
       </c>
       <c r="B715" s="8" t="inlineStr">
         <is>
-          <t>Dimaras</t>
+          <t>Schiller</t>
         </is>
       </c>
       <c r="C715" s="8" t="inlineStr">
         <is>
-          <t>Konstantinos</t>
+          <t>Christopher</t>
         </is>
       </c>
       <c r="D715" s="8" t="n">
@@ -35789,7 +35789,7 @@
       </c>
       <c r="I715" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Communication Arts</t>
         </is>
       </c>
       <c r="J715" s="8" t="n"/>
@@ -35801,16 +35801,16 @@
     </row>
     <row r="716">
       <c r="A716" s="8" t="n">
-        <v>117941</v>
+        <v>117998</v>
       </c>
       <c r="B716" s="8" t="inlineStr">
         <is>
-          <t>Schiller</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="C716" s="8" t="inlineStr">
         <is>
-          <t>Christopher</t>
+          <t>Charlie</t>
         </is>
       </c>
       <c r="D716" s="8" t="n">
@@ -35838,7 +35838,7 @@
       </c>
       <c r="I716" s="8" t="inlineStr">
         <is>
-          <t>Communication Arts</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J716" s="8" t="n"/>
@@ -35850,16 +35850,16 @@
     </row>
     <row r="717">
       <c r="A717" s="8" t="n">
-        <v>117998</v>
+        <v>118039</v>
       </c>
       <c r="B717" s="8" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Lazcano</t>
         </is>
       </c>
       <c r="C717" s="8" t="inlineStr">
         <is>
-          <t>Charlie</t>
+          <t>Alexander</t>
         </is>
       </c>
       <c r="D717" s="8" t="n">
@@ -35887,7 +35887,7 @@
       </c>
       <c r="I717" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J717" s="8" t="n"/>
@@ -35899,16 +35899,16 @@
     </row>
     <row r="718">
       <c r="A718" s="8" t="n">
-        <v>118039</v>
+        <v>118047</v>
       </c>
       <c r="B718" s="8" t="inlineStr">
         <is>
-          <t>Lazcano</t>
+          <t>Anastasopoulos</t>
         </is>
       </c>
       <c r="C718" s="8" t="inlineStr">
         <is>
-          <t>Alexander</t>
+          <t>Nikolas</t>
         </is>
       </c>
       <c r="D718" s="8" t="n">
@@ -35936,7 +35936,7 @@
       </c>
       <c r="I718" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J718" s="8" t="n"/>
@@ -35948,16 +35948,16 @@
     </row>
     <row r="719">
       <c r="A719" s="8" t="n">
-        <v>118047</v>
+        <v>118074</v>
       </c>
       <c r="B719" s="8" t="inlineStr">
         <is>
-          <t>Anastasopoulos</t>
+          <t>Russo-Felix</t>
         </is>
       </c>
       <c r="C719" s="8" t="inlineStr">
         <is>
-          <t>Nikolas</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="D719" s="8" t="n">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="I719" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J719" s="8" t="n"/>
@@ -35997,16 +35997,16 @@
     </row>
     <row r="720">
       <c r="A720" s="8" t="n">
-        <v>118074</v>
+        <v>118120</v>
       </c>
       <c r="B720" s="8" t="inlineStr">
         <is>
-          <t>Russo-Felix</t>
+          <t>Vincent</t>
         </is>
       </c>
       <c r="C720" s="8" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>John Paul</t>
         </is>
       </c>
       <c r="D720" s="8" t="n">
@@ -36034,7 +36034,7 @@
       </c>
       <c r="I720" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Theater</t>
         </is>
       </c>
       <c r="J720" s="8" t="n"/>
@@ -36046,16 +36046,16 @@
     </row>
     <row r="721">
       <c r="A721" s="8" t="n">
-        <v>118120</v>
+        <v>118143</v>
       </c>
       <c r="B721" s="8" t="inlineStr">
         <is>
-          <t>Vincent</t>
+          <t>Arcese</t>
         </is>
       </c>
       <c r="C721" s="8" t="inlineStr">
         <is>
-          <t>John Paul</t>
+          <t>Nico</t>
         </is>
       </c>
       <c r="D721" s="8" t="n">
@@ -36083,7 +36083,7 @@
       </c>
       <c r="I721" s="8" t="inlineStr">
         <is>
-          <t>Theater</t>
+          <t>Fine Arts</t>
         </is>
       </c>
       <c r="J721" s="8" t="n"/>
@@ -36095,16 +36095,16 @@
     </row>
     <row r="722">
       <c r="A722" s="8" t="n">
-        <v>118143</v>
+        <v>118181</v>
       </c>
       <c r="B722" s="8" t="inlineStr">
         <is>
-          <t>Arcese</t>
+          <t>Gill</t>
         </is>
       </c>
       <c r="C722" s="8" t="inlineStr">
         <is>
-          <t>Nico</t>
+          <t>Tariq</t>
         </is>
       </c>
       <c r="D722" s="8" t="n">
@@ -36132,7 +36132,7 @@
       </c>
       <c r="I722" s="8" t="inlineStr">
         <is>
-          <t>Fine Arts</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J722" s="8" t="n"/>
@@ -36144,20 +36144,20 @@
     </row>
     <row r="723">
       <c r="A723" s="8" t="n">
-        <v>118181</v>
+        <v>118186</v>
       </c>
       <c r="B723" s="8" t="inlineStr">
         <is>
-          <t>Gill</t>
+          <t>Fradette</t>
         </is>
       </c>
       <c r="C723" s="8" t="inlineStr">
         <is>
-          <t>Tariq</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="D723" s="8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E723" s="8" t="inlineStr">
         <is>
@@ -36181,7 +36181,7 @@
       </c>
       <c r="I723" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J723" s="8" t="n"/>
@@ -36193,20 +36193,20 @@
     </row>
     <row r="724">
       <c r="A724" s="8" t="n">
-        <v>118186</v>
+        <v>118189</v>
       </c>
       <c r="B724" s="8" t="inlineStr">
         <is>
-          <t>Fradette</t>
+          <t>Potenza</t>
         </is>
       </c>
       <c r="C724" s="8" t="inlineStr">
         <is>
-          <t>Nicholas</t>
+          <t>Charles</t>
         </is>
       </c>
       <c r="D724" s="8" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E724" s="8" t="inlineStr">
         <is>
@@ -36230,7 +36230,7 @@
       </c>
       <c r="I724" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J724" s="8" t="n"/>
@@ -36242,16 +36242,16 @@
     </row>
     <row r="725">
       <c r="A725" s="8" t="n">
-        <v>118189</v>
+        <v>118246</v>
       </c>
       <c r="B725" s="8" t="inlineStr">
         <is>
-          <t>Potenza</t>
+          <t>Mladenovic</t>
         </is>
       </c>
       <c r="C725" s="8" t="inlineStr">
         <is>
-          <t>Charles</t>
+          <t>Luka</t>
         </is>
       </c>
       <c r="D725" s="8" t="n">
@@ -36291,16 +36291,16 @@
     </row>
     <row r="726">
       <c r="A726" s="8" t="n">
-        <v>118246</v>
+        <v>118324</v>
       </c>
       <c r="B726" s="8" t="inlineStr">
         <is>
-          <t>Mladenovic</t>
+          <t>Semanczuk</t>
         </is>
       </c>
       <c r="C726" s="8" t="inlineStr">
         <is>
-          <t>Luka</t>
+          <t>Dean</t>
         </is>
       </c>
       <c r="D726" s="8" t="n">
@@ -36340,20 +36340,20 @@
     </row>
     <row r="727">
       <c r="A727" s="8" t="n">
-        <v>118324</v>
+        <v>118420</v>
       </c>
       <c r="B727" s="8" t="inlineStr">
         <is>
-          <t>Semanczuk</t>
+          <t>Bercovicz</t>
         </is>
       </c>
       <c r="C727" s="8" t="inlineStr">
         <is>
-          <t>Dean</t>
+          <t>Joseph</t>
         </is>
       </c>
       <c r="D727" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E727" s="8" t="inlineStr">
         <is>
@@ -36377,7 +36377,7 @@
       </c>
       <c r="I727" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J727" s="8" t="n"/>
@@ -36389,20 +36389,20 @@
     </row>
     <row r="728">
       <c r="A728" s="8" t="n">
-        <v>118420</v>
+        <v>118460</v>
       </c>
       <c r="B728" s="8" t="inlineStr">
         <is>
-          <t>Bercovicz</t>
+          <t>Coronel</t>
         </is>
       </c>
       <c r="C728" s="8" t="inlineStr">
         <is>
-          <t>Joseph</t>
+          <t>Mikalle</t>
         </is>
       </c>
       <c r="D728" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E728" s="8" t="inlineStr">
         <is>
@@ -36426,7 +36426,7 @@
       </c>
       <c r="I728" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="J728" s="8" t="n"/>
@@ -36438,16 +36438,16 @@
     </row>
     <row r="729">
       <c r="A729" s="8" t="n">
-        <v>118460</v>
+        <v>118533</v>
       </c>
       <c r="B729" s="8" t="inlineStr">
         <is>
-          <t>Coronel</t>
+          <t>Gallo</t>
         </is>
       </c>
       <c r="C729" s="8" t="inlineStr">
         <is>
-          <t>Mikalle</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="D729" s="8" t="n">
@@ -36475,7 +36475,7 @@
       </c>
       <c r="I729" s="8" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J729" s="8" t="n"/>
@@ -36487,16 +36487,16 @@
     </row>
     <row r="730">
       <c r="A730" s="8" t="n">
-        <v>118533</v>
+        <v>118565</v>
       </c>
       <c r="B730" s="8" t="inlineStr">
         <is>
-          <t>Gallo</t>
+          <t>Hauck</t>
         </is>
       </c>
       <c r="C730" s="8" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>David</t>
         </is>
       </c>
       <c r="D730" s="8" t="n">
@@ -36536,16 +36536,16 @@
     </row>
     <row r="731">
       <c r="A731" s="8" t="n">
-        <v>118565</v>
+        <v>118601</v>
       </c>
       <c r="B731" s="8" t="inlineStr">
         <is>
-          <t>Hauck</t>
+          <t>Torres</t>
         </is>
       </c>
       <c r="C731" s="8" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Calvin</t>
         </is>
       </c>
       <c r="D731" s="8" t="n">
@@ -36573,7 +36573,7 @@
       </c>
       <c r="I731" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J731" s="8" t="n"/>
@@ -36585,16 +36585,16 @@
     </row>
     <row r="732">
       <c r="A732" s="8" t="n">
-        <v>118601</v>
+        <v>118635</v>
       </c>
       <c r="B732" s="8" t="inlineStr">
         <is>
-          <t>Torres</t>
+          <t>Carey</t>
         </is>
       </c>
       <c r="C732" s="8" t="inlineStr">
         <is>
-          <t>Calvin</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="D732" s="8" t="n">
@@ -36622,7 +36622,7 @@
       </c>
       <c r="I732" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J732" s="8" t="n"/>
@@ -36634,16 +36634,16 @@
     </row>
     <row r="733">
       <c r="A733" s="8" t="n">
-        <v>118635</v>
+        <v>118775</v>
       </c>
       <c r="B733" s="8" t="inlineStr">
         <is>
-          <t>Carey</t>
+          <t>Hollenback</t>
         </is>
       </c>
       <c r="C733" s="8" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Liam</t>
         </is>
       </c>
       <c r="D733" s="8" t="n">
@@ -36671,7 +36671,7 @@
       </c>
       <c r="I733" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Theater</t>
         </is>
       </c>
       <c r="J733" s="8" t="n"/>
@@ -36683,16 +36683,16 @@
     </row>
     <row r="734">
       <c r="A734" s="8" t="n">
-        <v>118775</v>
+        <v>118815</v>
       </c>
       <c r="B734" s="8" t="inlineStr">
         <is>
-          <t>Hollenback</t>
+          <t>Agosti</t>
         </is>
       </c>
       <c r="C734" s="8" t="inlineStr">
         <is>
-          <t>Liam</t>
+          <t>Andrew</t>
         </is>
       </c>
       <c r="D734" s="8" t="n">
@@ -36720,7 +36720,7 @@
       </c>
       <c r="I734" s="8" t="inlineStr">
         <is>
-          <t>Theater</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J734" s="8" t="n"/>
@@ -36732,16 +36732,16 @@
     </row>
     <row r="735">
       <c r="A735" s="8" t="n">
-        <v>118815</v>
+        <v>118828</v>
       </c>
       <c r="B735" s="8" t="inlineStr">
         <is>
-          <t>Agosti</t>
+          <t>McSharry</t>
         </is>
       </c>
       <c r="C735" s="8" t="inlineStr">
         <is>
-          <t>Andrew</t>
+          <t>Kyle</t>
         </is>
       </c>
       <c r="D735" s="8" t="n">
@@ -36781,16 +36781,16 @@
     </row>
     <row r="736">
       <c r="A736" s="8" t="n">
-        <v>118828</v>
+        <v>118849</v>
       </c>
       <c r="B736" s="8" t="inlineStr">
         <is>
-          <t>McSharry</t>
+          <t>Contreras</t>
         </is>
       </c>
       <c r="C736" s="8" t="inlineStr">
         <is>
-          <t>Kyle</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="D736" s="8" t="n">
@@ -36830,16 +36830,16 @@
     </row>
     <row r="737">
       <c r="A737" s="8" t="n">
-        <v>118849</v>
+        <v>118861</v>
       </c>
       <c r="B737" s="8" t="inlineStr">
         <is>
-          <t>Contreras</t>
+          <t>Abdrabboh</t>
         </is>
       </c>
       <c r="C737" s="8" t="inlineStr">
         <is>
-          <t>Nicholas</t>
+          <t>Rizk</t>
         </is>
       </c>
       <c r="D737" s="8" t="n">
@@ -36879,16 +36879,16 @@
     </row>
     <row r="738">
       <c r="A738" s="8" t="n">
-        <v>118861</v>
+        <v>118889</v>
       </c>
       <c r="B738" s="8" t="inlineStr">
         <is>
-          <t>Abdrabboh</t>
+          <t>Désiré</t>
         </is>
       </c>
       <c r="C738" s="8" t="inlineStr">
         <is>
-          <t>Rizk</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="D738" s="8" t="n">
@@ -36916,7 +36916,7 @@
       </c>
       <c r="I738" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J738" s="8" t="n"/>
@@ -36928,16 +36928,16 @@
     </row>
     <row r="739">
       <c r="A739" s="8" t="n">
-        <v>118889</v>
+        <v>118902</v>
       </c>
       <c r="B739" s="8" t="inlineStr">
         <is>
-          <t>Désiré</t>
+          <t>Cavagnaro</t>
         </is>
       </c>
       <c r="C739" s="8" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="D739" s="8" t="n">
@@ -36965,7 +36965,7 @@
       </c>
       <c r="I739" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J739" s="8" t="n"/>
@@ -36977,20 +36977,20 @@
     </row>
     <row r="740">
       <c r="A740" s="8" t="n">
-        <v>118902</v>
+        <v>119012</v>
       </c>
       <c r="B740" s="8" t="inlineStr">
         <is>
-          <t>Cavagnaro</t>
+          <t>Zapata</t>
         </is>
       </c>
       <c r="C740" s="8" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Pascual</t>
         </is>
       </c>
       <c r="D740" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E740" s="8" t="inlineStr">
         <is>
@@ -37009,12 +37009,12 @@
       </c>
       <c r="H740" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I740" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J740" s="8" t="n"/>
@@ -37026,20 +37026,20 @@
     </row>
     <row r="741">
       <c r="A741" s="8" t="n">
-        <v>119012</v>
+        <v>119020</v>
       </c>
       <c r="B741" s="8" t="inlineStr">
         <is>
-          <t>Zapata</t>
+          <t>Cyckowski</t>
         </is>
       </c>
       <c r="C741" s="8" t="inlineStr">
         <is>
-          <t>Pascual</t>
+          <t>Sean</t>
         </is>
       </c>
       <c r="D741" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E741" s="8" t="inlineStr">
         <is>
@@ -37058,12 +37058,12 @@
       </c>
       <c r="H741" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I741" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J741" s="8" t="n"/>
@@ -37075,16 +37075,16 @@
     </row>
     <row r="742">
       <c r="A742" s="8" t="n">
-        <v>119020</v>
+        <v>119104</v>
       </c>
       <c r="B742" s="8" t="inlineStr">
         <is>
-          <t>Cyckowski</t>
+          <t>Howell</t>
         </is>
       </c>
       <c r="C742" s="8" t="inlineStr">
         <is>
-          <t>Sean</t>
+          <t>Jaxon</t>
         </is>
       </c>
       <c r="D742" s="8" t="n">
@@ -37124,16 +37124,16 @@
     </row>
     <row r="743">
       <c r="A743" s="8" t="n">
-        <v>119104</v>
+        <v>119190</v>
       </c>
       <c r="B743" s="8" t="inlineStr">
         <is>
-          <t>Howell</t>
+          <t>Ortiz</t>
         </is>
       </c>
       <c r="C743" s="8" t="inlineStr">
         <is>
-          <t>Jaxon</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="D743" s="8" t="n">
@@ -37173,16 +37173,16 @@
     </row>
     <row r="744">
       <c r="A744" s="8" t="n">
-        <v>119190</v>
+        <v>119257</v>
       </c>
       <c r="B744" s="8" t="inlineStr">
         <is>
-          <t>Ortiz</t>
+          <t>Lopez</t>
         </is>
       </c>
       <c r="C744" s="8" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Liam</t>
         </is>
       </c>
       <c r="D744" s="8" t="n">
@@ -37210,7 +37210,7 @@
       </c>
       <c r="I744" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>Fine Arts</t>
         </is>
       </c>
       <c r="J744" s="8" t="n"/>
@@ -37222,16 +37222,16 @@
     </row>
     <row r="745">
       <c r="A745" s="8" t="n">
-        <v>119257</v>
+        <v>119307</v>
       </c>
       <c r="B745" s="8" t="inlineStr">
         <is>
-          <t>Lopez</t>
+          <t>Scolaro</t>
         </is>
       </c>
       <c r="C745" s="8" t="inlineStr">
         <is>
-          <t>Liam</t>
+          <t>Sebastian-Jon</t>
         </is>
       </c>
       <c r="D745" s="8" t="n">
@@ -37271,16 +37271,16 @@
     </row>
     <row r="746">
       <c r="A746" s="8" t="n">
-        <v>119307</v>
+        <v>119312</v>
       </c>
       <c r="B746" s="8" t="inlineStr">
         <is>
-          <t>Scolaro</t>
+          <t>Cassano</t>
         </is>
       </c>
       <c r="C746" s="8" t="inlineStr">
         <is>
-          <t>Sebastian-Jon</t>
+          <t>Alexander</t>
         </is>
       </c>
       <c r="D746" s="8" t="n">
@@ -37308,7 +37308,7 @@
       </c>
       <c r="I746" s="8" t="inlineStr">
         <is>
-          <t>Fine Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J746" s="8" t="n"/>
@@ -37320,16 +37320,16 @@
     </row>
     <row r="747">
       <c r="A747" s="8" t="n">
-        <v>119312</v>
+        <v>119360</v>
       </c>
       <c r="B747" s="8" t="inlineStr">
         <is>
-          <t>Cassano</t>
+          <t>Doyle</t>
         </is>
       </c>
       <c r="C747" s="8" t="inlineStr">
         <is>
-          <t>Alexander</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="D747" s="8" t="n">
@@ -37357,7 +37357,7 @@
       </c>
       <c r="I747" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J747" s="8" t="n"/>
@@ -37369,20 +37369,20 @@
     </row>
     <row r="748">
       <c r="A748" s="8" t="n">
-        <v>119360</v>
+        <v>119384</v>
       </c>
       <c r="B748" s="8" t="inlineStr">
         <is>
-          <t>Doyle</t>
+          <t>Clarke-Richardson</t>
         </is>
       </c>
       <c r="C748" s="8" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Cayden</t>
         </is>
       </c>
       <c r="D748" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E748" s="8" t="inlineStr">
         <is>
@@ -37418,20 +37418,20 @@
     </row>
     <row r="749">
       <c r="A749" s="8" t="n">
-        <v>119384</v>
+        <v>119397</v>
       </c>
       <c r="B749" s="8" t="inlineStr">
         <is>
-          <t>Clarke-Richardson</t>
+          <t>O’Connor</t>
         </is>
       </c>
       <c r="C749" s="8" t="inlineStr">
         <is>
-          <t>Cayden</t>
+          <t>Mason</t>
         </is>
       </c>
       <c r="D749" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E749" s="8" t="inlineStr">
         <is>
@@ -37455,7 +37455,7 @@
       </c>
       <c r="I749" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Communication Arts</t>
         </is>
       </c>
       <c r="J749" s="8" t="n"/>
@@ -37467,20 +37467,20 @@
     </row>
     <row r="750">
       <c r="A750" s="8" t="n">
-        <v>119397</v>
+        <v>119400</v>
       </c>
       <c r="B750" s="8" t="inlineStr">
         <is>
-          <t>O’Connor</t>
+          <t>Pavone</t>
         </is>
       </c>
       <c r="C750" s="8" t="inlineStr">
         <is>
-          <t>Mason</t>
+          <t>Anthony</t>
         </is>
       </c>
       <c r="D750" s="8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E750" s="8" t="inlineStr">
         <is>
@@ -37504,7 +37504,7 @@
       </c>
       <c r="I750" s="8" t="inlineStr">
         <is>
-          <t>Communication Arts</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J750" s="8" t="n"/>
@@ -37516,20 +37516,20 @@
     </row>
     <row r="751">
       <c r="A751" s="8" t="n">
-        <v>119400</v>
+        <v>119412</v>
       </c>
       <c r="B751" s="8" t="inlineStr">
         <is>
-          <t>Pavone</t>
+          <t>Reidy</t>
         </is>
       </c>
       <c r="C751" s="8" t="inlineStr">
         <is>
-          <t>Anthony</t>
+          <t>Sean</t>
         </is>
       </c>
       <c r="D751" s="8" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E751" s="8" t="inlineStr">
         <is>
@@ -37553,7 +37553,7 @@
       </c>
       <c r="I751" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J751" s="8" t="n"/>
@@ -37565,16 +37565,16 @@
     </row>
     <row r="752">
       <c r="A752" s="8" t="n">
-        <v>119412</v>
+        <v>119418</v>
       </c>
       <c r="B752" s="8" t="inlineStr">
         <is>
-          <t>Reidy</t>
+          <t>Felix</t>
         </is>
       </c>
       <c r="C752" s="8" t="inlineStr">
         <is>
-          <t>Sean</t>
+          <t>Victor</t>
         </is>
       </c>
       <c r="D752" s="8" t="n">
@@ -37602,7 +37602,7 @@
       </c>
       <c r="I752" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Computer Science</t>
         </is>
       </c>
       <c r="J752" s="8" t="n"/>
@@ -37614,16 +37614,16 @@
     </row>
     <row r="753">
       <c r="A753" s="8" t="n">
-        <v>119418</v>
+        <v>119466</v>
       </c>
       <c r="B753" s="8" t="inlineStr">
         <is>
-          <t>Felix</t>
+          <t>Medyan</t>
         </is>
       </c>
       <c r="C753" s="8" t="inlineStr">
         <is>
-          <t>Victor</t>
+          <t>Adam</t>
         </is>
       </c>
       <c r="D753" s="8" t="n">
@@ -37651,7 +37651,7 @@
       </c>
       <c r="I753" s="8" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J753" s="8" t="n"/>
@@ -37663,16 +37663,16 @@
     </row>
     <row r="754">
       <c r="A754" s="8" t="n">
-        <v>119466</v>
+        <v>119498</v>
       </c>
       <c r="B754" s="8" t="inlineStr">
         <is>
-          <t>Medyan</t>
+          <t>Rodriguez</t>
         </is>
       </c>
       <c r="C754" s="8" t="inlineStr">
         <is>
-          <t>Adam</t>
+          <t>Pedro</t>
         </is>
       </c>
       <c r="D754" s="8" t="n">
@@ -37700,7 +37700,7 @@
       </c>
       <c r="I754" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J754" s="8" t="n"/>
@@ -37712,20 +37712,20 @@
     </row>
     <row r="755">
       <c r="A755" s="8" t="n">
-        <v>119498</v>
+        <v>119514</v>
       </c>
       <c r="B755" s="8" t="inlineStr">
         <is>
-          <t>Rodriguez</t>
+          <t>Roemer</t>
         </is>
       </c>
       <c r="C755" s="8" t="inlineStr">
         <is>
-          <t>Pedro</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="D755" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E755" s="8" t="inlineStr">
         <is>
@@ -37749,7 +37749,7 @@
       </c>
       <c r="I755" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J755" s="8" t="n"/>
@@ -37761,20 +37761,20 @@
     </row>
     <row r="756">
       <c r="A756" s="8" t="n">
-        <v>119514</v>
+        <v>119589</v>
       </c>
       <c r="B756" s="8" t="inlineStr">
         <is>
-          <t>Roemer</t>
+          <t>Martinez</t>
         </is>
       </c>
       <c r="C756" s="8" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="D756" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E756" s="8" t="inlineStr">
         <is>
@@ -37798,7 +37798,7 @@
       </c>
       <c r="I756" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J756" s="8" t="n"/>
@@ -37810,20 +37810,20 @@
     </row>
     <row r="757">
       <c r="A757" s="8" t="n">
-        <v>119589</v>
+        <v>119656</v>
       </c>
       <c r="B757" s="8" t="inlineStr">
         <is>
-          <t>Martinez</t>
+          <t>Pierce</t>
         </is>
       </c>
       <c r="C757" s="8" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Dylan</t>
         </is>
       </c>
       <c r="D757" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E757" s="8" t="inlineStr">
         <is>
@@ -37847,7 +37847,7 @@
       </c>
       <c r="I757" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J757" s="8" t="n"/>
@@ -37859,16 +37859,16 @@
     </row>
     <row r="758">
       <c r="A758" s="8" t="n">
-        <v>119656</v>
+        <v>119659</v>
       </c>
       <c r="B758" s="8" t="inlineStr">
         <is>
-          <t>Pierce</t>
+          <t>Altieri</t>
         </is>
       </c>
       <c r="C758" s="8" t="inlineStr">
         <is>
-          <t>Dylan</t>
+          <t>Joseph</t>
         </is>
       </c>
       <c r="D758" s="8" t="n">
@@ -37908,20 +37908,20 @@
     </row>
     <row r="759">
       <c r="A759" s="8" t="n">
-        <v>119659</v>
+        <v>119737</v>
       </c>
       <c r="B759" s="8" t="inlineStr">
         <is>
-          <t>Altieri</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="C759" s="8" t="inlineStr">
         <is>
-          <t>Joseph</t>
+          <t>Karter</t>
         </is>
       </c>
       <c r="D759" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E759" s="8" t="inlineStr">
         <is>
@@ -37945,7 +37945,7 @@
       </c>
       <c r="I759" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J759" s="8" t="n"/>
@@ -37957,16 +37957,16 @@
     </row>
     <row r="760">
       <c r="A760" s="8" t="n">
-        <v>119737</v>
+        <v>119950</v>
       </c>
       <c r="B760" s="8" t="inlineStr">
         <is>
-          <t>Taylor</t>
+          <t>Mims</t>
         </is>
       </c>
       <c r="C760" s="8" t="inlineStr">
         <is>
-          <t>Karter</t>
+          <t>Davion</t>
         </is>
       </c>
       <c r="D760" s="8" t="n">
@@ -37994,7 +37994,7 @@
       </c>
       <c r="I760" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J760" s="8" t="n"/>
@@ -38006,16 +38006,16 @@
     </row>
     <row r="761">
       <c r="A761" s="8" t="n">
-        <v>119950</v>
+        <v>119966</v>
       </c>
       <c r="B761" s="8" t="inlineStr">
         <is>
-          <t>Mims</t>
+          <t>Varley</t>
         </is>
       </c>
       <c r="C761" s="8" t="inlineStr">
         <is>
-          <t>Davion</t>
+          <t>Seamus</t>
         </is>
       </c>
       <c r="D761" s="8" t="n">
@@ -38043,7 +38043,7 @@
       </c>
       <c r="I761" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J761" s="8" t="n"/>
@@ -38055,16 +38055,16 @@
     </row>
     <row r="762">
       <c r="A762" s="8" t="n">
-        <v>119966</v>
+        <v>120024</v>
       </c>
       <c r="B762" s="8" t="inlineStr">
         <is>
-          <t>Varley</t>
+          <t>Jimmy Thomas</t>
         </is>
       </c>
       <c r="C762" s="8" t="inlineStr">
         <is>
-          <t>Seamus</t>
+          <t>Jake</t>
         </is>
       </c>
       <c r="D762" s="8" t="n">
@@ -38092,7 +38092,7 @@
       </c>
       <c r="I762" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J762" s="8" t="n"/>
@@ -38104,16 +38104,16 @@
     </row>
     <row r="763">
       <c r="A763" s="8" t="n">
-        <v>120024</v>
+        <v>120047</v>
       </c>
       <c r="B763" s="8" t="inlineStr">
         <is>
-          <t>Jimmy Thomas</t>
+          <t>Daskaloski</t>
         </is>
       </c>
       <c r="C763" s="8" t="inlineStr">
         <is>
-          <t>Jake</t>
+          <t>Darian</t>
         </is>
       </c>
       <c r="D763" s="8" t="n">
@@ -38141,7 +38141,7 @@
       </c>
       <c r="I763" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J763" s="8" t="n"/>
@@ -38153,16 +38153,16 @@
     </row>
     <row r="764">
       <c r="A764" s="8" t="n">
-        <v>120047</v>
+        <v>120053</v>
       </c>
       <c r="B764" s="8" t="inlineStr">
         <is>
-          <t>Daskaloski</t>
+          <t>Robinson</t>
         </is>
       </c>
       <c r="C764" s="8" t="inlineStr">
         <is>
-          <t>Darian</t>
+          <t>Tyler</t>
         </is>
       </c>
       <c r="D764" s="8" t="n">
@@ -38190,7 +38190,7 @@
       </c>
       <c r="I764" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Fine Arts</t>
         </is>
       </c>
       <c r="J764" s="8" t="n"/>
@@ -38202,16 +38202,16 @@
     </row>
     <row r="765">
       <c r="A765" s="8" t="n">
-        <v>120053</v>
+        <v>120069</v>
       </c>
       <c r="B765" s="8" t="inlineStr">
         <is>
-          <t>Robinson</t>
+          <t>Ortiz</t>
         </is>
       </c>
       <c r="C765" s="8" t="inlineStr">
         <is>
-          <t>Tyler</t>
+          <t>Evan</t>
         </is>
       </c>
       <c r="D765" s="8" t="n">
@@ -38239,7 +38239,7 @@
       </c>
       <c r="I765" s="8" t="inlineStr">
         <is>
-          <t>Fine Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J765" s="8" t="n"/>
@@ -38251,16 +38251,16 @@
     </row>
     <row r="766">
       <c r="A766" s="8" t="n">
-        <v>120069</v>
+        <v>120089</v>
       </c>
       <c r="B766" s="8" t="inlineStr">
         <is>
-          <t>Ortiz</t>
+          <t>Palanca</t>
         </is>
       </c>
       <c r="C766" s="8" t="inlineStr">
         <is>
-          <t>Evan</t>
+          <t>Cassius</t>
         </is>
       </c>
       <c r="D766" s="8" t="n">
@@ -38300,16 +38300,16 @@
     </row>
     <row r="767">
       <c r="A767" s="8" t="n">
-        <v>120089</v>
+        <v>120126</v>
       </c>
       <c r="B767" s="8" t="inlineStr">
         <is>
-          <t>Palanca</t>
+          <t>Lores</t>
         </is>
       </c>
       <c r="C767" s="8" t="inlineStr">
         <is>
-          <t>Cassius</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="D767" s="8" t="n">
@@ -38349,16 +38349,16 @@
     </row>
     <row r="768">
       <c r="A768" s="8" t="n">
-        <v>120126</v>
+        <v>120187</v>
       </c>
       <c r="B768" s="8" t="inlineStr">
         <is>
-          <t>Lores</t>
+          <t>Perno</t>
         </is>
       </c>
       <c r="C768" s="8" t="inlineStr">
         <is>
-          <t>Nicholas</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="D768" s="8" t="n">
@@ -38398,16 +38398,16 @@
     </row>
     <row r="769">
       <c r="A769" s="8" t="n">
-        <v>120187</v>
+        <v>120211</v>
       </c>
       <c r="B769" s="8" t="inlineStr">
         <is>
-          <t>Perno</t>
+          <t>Ji</t>
         </is>
       </c>
       <c r="C769" s="8" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Changjun</t>
         </is>
       </c>
       <c r="D769" s="8" t="n">
@@ -38447,16 +38447,16 @@
     </row>
     <row r="770">
       <c r="A770" s="8" t="n">
-        <v>120211</v>
+        <v>120240</v>
       </c>
       <c r="B770" s="8" t="inlineStr">
         <is>
-          <t>Ji</t>
+          <t>Kearns</t>
         </is>
       </c>
       <c r="C770" s="8" t="inlineStr">
         <is>
-          <t>Changjun</t>
+          <t>Nolan</t>
         </is>
       </c>
       <c r="D770" s="8" t="n">
@@ -38496,16 +38496,16 @@
     </row>
     <row r="771">
       <c r="A771" s="8" t="n">
-        <v>120240</v>
+        <v>120267</v>
       </c>
       <c r="B771" s="8" t="inlineStr">
         <is>
-          <t>Kearns</t>
+          <t>Perruso</t>
         </is>
       </c>
       <c r="C771" s="8" t="inlineStr">
         <is>
-          <t>Nolan</t>
+          <t>Jayden</t>
         </is>
       </c>
       <c r="D771" s="8" t="n">
@@ -38533,7 +38533,7 @@
       </c>
       <c r="I771" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Fine Arts</t>
         </is>
       </c>
       <c r="J771" s="8" t="n"/>
@@ -38545,16 +38545,16 @@
     </row>
     <row r="772">
       <c r="A772" s="8" t="n">
-        <v>120267</v>
+        <v>120279</v>
       </c>
       <c r="B772" s="8" t="inlineStr">
         <is>
-          <t>Perruso</t>
+          <t>Pytel</t>
         </is>
       </c>
       <c r="C772" s="8" t="inlineStr">
         <is>
-          <t>Jayden</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="D772" s="8" t="n">
@@ -38582,7 +38582,7 @@
       </c>
       <c r="I772" s="8" t="inlineStr">
         <is>
-          <t>Fine Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J772" s="8" t="n"/>
@@ -38594,16 +38594,16 @@
     </row>
     <row r="773">
       <c r="A773" s="8" t="n">
-        <v>120279</v>
+        <v>120374</v>
       </c>
       <c r="B773" s="8" t="inlineStr">
         <is>
-          <t>Pytel</t>
+          <t>Ferron</t>
         </is>
       </c>
       <c r="C773" s="8" t="inlineStr">
         <is>
-          <t>Nicholas</t>
+          <t>Jeremiah</t>
         </is>
       </c>
       <c r="D773" s="8" t="n">
@@ -38626,12 +38626,12 @@
       </c>
       <c r="H773" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I773" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J773" s="8" t="n"/>
@@ -38643,16 +38643,16 @@
     </row>
     <row r="774">
       <c r="A774" s="8" t="n">
-        <v>120374</v>
+        <v>120399</v>
       </c>
       <c r="B774" s="8" t="inlineStr">
         <is>
-          <t>Ferron</t>
+          <t>Katariya</t>
         </is>
       </c>
       <c r="C774" s="8" t="inlineStr">
         <is>
-          <t>Jeremiah</t>
+          <t>Ayush</t>
         </is>
       </c>
       <c r="D774" s="8" t="n">
@@ -38675,12 +38675,12 @@
       </c>
       <c r="H774" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I774" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J774" s="8" t="n"/>
@@ -38692,16 +38692,16 @@
     </row>
     <row r="775">
       <c r="A775" s="8" t="n">
-        <v>120399</v>
+        <v>120418</v>
       </c>
       <c r="B775" s="8" t="inlineStr">
         <is>
-          <t>Katariya</t>
+          <t>Khan</t>
         </is>
       </c>
       <c r="C775" s="8" t="inlineStr">
         <is>
-          <t>Ayush</t>
+          <t>Evan</t>
         </is>
       </c>
       <c r="D775" s="8" t="n">
@@ -38741,16 +38741,16 @@
     </row>
     <row r="776">
       <c r="A776" s="8" t="n">
-        <v>120418</v>
+        <v>120492</v>
       </c>
       <c r="B776" s="8" t="inlineStr">
         <is>
-          <t>Khan</t>
+          <t>Winborne</t>
         </is>
       </c>
       <c r="C776" s="8" t="inlineStr">
         <is>
-          <t>Evan</t>
+          <t>Jayce</t>
         </is>
       </c>
       <c r="D776" s="8" t="n">
@@ -38790,20 +38790,20 @@
     </row>
     <row r="777">
       <c r="A777" s="8" t="n">
-        <v>120492</v>
+        <v>120546</v>
       </c>
       <c r="B777" s="8" t="inlineStr">
         <is>
-          <t>Winborne</t>
+          <t>Williams</t>
         </is>
       </c>
       <c r="C777" s="8" t="inlineStr">
         <is>
-          <t>Jayce</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="D777" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E777" s="8" t="inlineStr">
         <is>
@@ -38827,7 +38827,7 @@
       </c>
       <c r="I777" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J777" s="8" t="n"/>
@@ -38839,20 +38839,20 @@
     </row>
     <row r="778">
       <c r="A778" s="8" t="n">
-        <v>120546</v>
+        <v>120587</v>
       </c>
       <c r="B778" s="8" t="inlineStr">
         <is>
-          <t>Williams</t>
+          <t>Nowobilski-Doyle</t>
         </is>
       </c>
       <c r="C778" s="8" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Sean</t>
         </is>
       </c>
       <c r="D778" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E778" s="8" t="inlineStr">
         <is>
@@ -38876,7 +38876,7 @@
       </c>
       <c r="I778" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J778" s="8" t="n"/>
@@ -38888,16 +38888,16 @@
     </row>
     <row r="779">
       <c r="A779" s="8" t="n">
-        <v>120587</v>
+        <v>120645</v>
       </c>
       <c r="B779" s="8" t="inlineStr">
         <is>
-          <t>Nowobilski-Doyle</t>
+          <t>Swenson</t>
         </is>
       </c>
       <c r="C779" s="8" t="inlineStr">
         <is>
-          <t>Sean</t>
+          <t>Russell</t>
         </is>
       </c>
       <c r="D779" s="8" t="n">
@@ -38925,7 +38925,7 @@
       </c>
       <c r="I779" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J779" s="8" t="n"/>
@@ -38937,16 +38937,16 @@
     </row>
     <row r="780">
       <c r="A780" s="8" t="n">
-        <v>120645</v>
+        <v>120664</v>
       </c>
       <c r="B780" s="8" t="inlineStr">
         <is>
-          <t>Swenson</t>
+          <t>Marcazo</t>
         </is>
       </c>
       <c r="C780" s="8" t="inlineStr">
         <is>
-          <t>Russell</t>
+          <t>Anthony</t>
         </is>
       </c>
       <c r="D780" s="8" t="n">
@@ -38986,16 +38986,16 @@
     </row>
     <row r="781">
       <c r="A781" s="8" t="n">
-        <v>120664</v>
+        <v>120688</v>
       </c>
       <c r="B781" s="8" t="inlineStr">
         <is>
-          <t>Marcazo</t>
+          <t>Ruiter</t>
         </is>
       </c>
       <c r="C781" s="8" t="inlineStr">
         <is>
-          <t>Anthony</t>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="D781" s="8" t="n">
@@ -39034,48 +39034,48 @@
       </c>
     </row>
     <row r="782">
-      <c r="A782" s="8" t="n">
-        <v>120688</v>
-      </c>
-      <c r="B782" s="8" t="inlineStr">
-        <is>
-          <t>Ruiter</t>
-        </is>
-      </c>
-      <c r="C782" s="8" t="inlineStr">
-        <is>
-          <t>Ryan</t>
-        </is>
-      </c>
-      <c r="D782" s="8" t="n">
+      <c r="A782" s="11" t="n">
+        <v>120718</v>
+      </c>
+      <c r="B782" s="16" t="inlineStr">
+        <is>
+          <t>Myers</t>
+        </is>
+      </c>
+      <c r="C782" s="16" t="inlineStr">
+        <is>
+          <t>Charles</t>
+        </is>
+      </c>
+      <c r="D782" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="E782" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F782" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G782" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H782" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I782" s="8" t="inlineStr">
+      <c r="E782" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F782" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G782" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H782" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I782" s="10" t="inlineStr">
         <is>
           <t>Business</t>
         </is>
       </c>
-      <c r="J782" s="8" t="n"/>
+      <c r="J782" s="9" t="n"/>
       <c r="K782" s="8" t="inlineStr">
         <is>
           <t>N</t>
@@ -39083,48 +39083,48 @@
       </c>
     </row>
     <row r="783">
-      <c r="A783" s="11" t="n">
-        <v>120718</v>
-      </c>
-      <c r="B783" s="16" t="inlineStr">
-        <is>
-          <t>Myers</t>
-        </is>
-      </c>
-      <c r="C783" s="16" t="inlineStr">
-        <is>
-          <t>Charles</t>
-        </is>
-      </c>
-      <c r="D783" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="E783" s="10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F783" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G783" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H783" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I783" s="10" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="J783" s="9" t="n"/>
+      <c r="A783" s="8" t="n">
+        <v>120834</v>
+      </c>
+      <c r="B783" s="8" t="inlineStr">
+        <is>
+          <t>McNeal</t>
+        </is>
+      </c>
+      <c r="C783" s="8" t="inlineStr">
+        <is>
+          <t>Harlem</t>
+        </is>
+      </c>
+      <c r="D783" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E783" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F783" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G783" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H783" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I783" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J783" s="8" t="n"/>
       <c r="K783" s="8" t="inlineStr">
         <is>
           <t>N</t>
@@ -39133,20 +39133,20 @@
     </row>
     <row r="784">
       <c r="A784" s="8" t="n">
-        <v>120834</v>
+        <v>120899</v>
       </c>
       <c r="B784" s="8" t="inlineStr">
         <is>
-          <t>McNeal</t>
+          <t>Kornacki</t>
         </is>
       </c>
       <c r="C784" s="8" t="inlineStr">
         <is>
-          <t>Harlem</t>
+          <t>Conrad</t>
         </is>
       </c>
       <c r="D784" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E784" s="8" t="inlineStr">
         <is>
@@ -39170,7 +39170,7 @@
       </c>
       <c r="I784" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J784" s="8" t="n"/>
@@ -39181,17 +39181,17 @@
       </c>
     </row>
     <row r="785">
-      <c r="A785" s="8" t="n">
-        <v>120899</v>
-      </c>
-      <c r="B785" s="8" t="inlineStr">
-        <is>
-          <t>Kornacki</t>
-        </is>
-      </c>
-      <c r="C785" s="8" t="inlineStr">
-        <is>
-          <t>Conrad</t>
+      <c r="A785" s="20" t="n">
+        <v>120940</v>
+      </c>
+      <c r="B785" s="19" t="inlineStr">
+        <is>
+          <t>Sidibe</t>
+        </is>
+      </c>
+      <c r="C785" s="19" t="inlineStr">
+        <is>
+          <t>Mohamed</t>
         </is>
       </c>
       <c r="D785" s="8" t="n">
@@ -39230,17 +39230,19 @@
       </c>
     </row>
     <row r="786">
-      <c r="A786" s="20" t="n">
-        <v>120940</v>
-      </c>
-      <c r="B786" s="19" t="inlineStr">
-        <is>
-          <t>Sidibe</t>
-        </is>
-      </c>
-      <c r="C786" s="19" t="inlineStr">
-        <is>
-          <t>Mohamed</t>
+      <c r="A786" s="8" t="inlineStr">
+        <is>
+          <t>121012</t>
+        </is>
+      </c>
+      <c r="B786" s="8" t="inlineStr">
+        <is>
+          <t>Garcia</t>
+        </is>
+      </c>
+      <c r="C786" s="8" t="inlineStr">
+        <is>
+          <t>Jace Jaden</t>
         </is>
       </c>
       <c r="D786" s="8" t="n">
@@ -39268,7 +39270,7 @@
       </c>
       <c r="I786" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="J786" s="8" t="n"/>
@@ -39279,23 +39281,21 @@
       </c>
     </row>
     <row r="787">
-      <c r="A787" s="8" t="inlineStr">
-        <is>
-          <t>121012</t>
-        </is>
+      <c r="A787" s="8" t="n">
+        <v>121020</v>
       </c>
       <c r="B787" s="8" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Pulgarin</t>
         </is>
       </c>
       <c r="C787" s="8" t="inlineStr">
         <is>
-          <t>Jace Jaden</t>
+          <t>Cesar</t>
         </is>
       </c>
       <c r="D787" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E787" s="8" t="inlineStr">
         <is>
@@ -39319,7 +39319,7 @@
       </c>
       <c r="I787" s="8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J787" s="8" t="n"/>
@@ -39331,20 +39331,20 @@
     </row>
     <row r="788">
       <c r="A788" s="8" t="n">
-        <v>121020</v>
+        <v>121117</v>
       </c>
       <c r="B788" s="8" t="inlineStr">
         <is>
-          <t>Pulgarin</t>
+          <t>Motylinski</t>
         </is>
       </c>
       <c r="C788" s="8" t="inlineStr">
         <is>
-          <t>Cesar</t>
+          <t>Ludovic</t>
         </is>
       </c>
       <c r="D788" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E788" s="8" t="inlineStr">
         <is>
@@ -39368,7 +39368,7 @@
       </c>
       <c r="I788" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J788" s="8" t="n"/>
@@ -39380,20 +39380,20 @@
     </row>
     <row r="789">
       <c r="A789" s="8" t="n">
-        <v>121117</v>
+        <v>121187</v>
       </c>
       <c r="B789" s="8" t="inlineStr">
         <is>
-          <t>Motylinski</t>
+          <t>Sokol</t>
         </is>
       </c>
       <c r="C789" s="8" t="inlineStr">
         <is>
-          <t>Ludovic</t>
+          <t>Jacob</t>
         </is>
       </c>
       <c r="D789" s="8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E789" s="8" t="inlineStr">
         <is>
@@ -39429,20 +39429,20 @@
     </row>
     <row r="790">
       <c r="A790" s="8" t="n">
-        <v>121187</v>
+        <v>121196</v>
       </c>
       <c r="B790" s="8" t="inlineStr">
         <is>
-          <t>Sokol</t>
+          <t>Bocchino</t>
         </is>
       </c>
       <c r="C790" s="8" t="inlineStr">
         <is>
-          <t>Jacob</t>
+          <t>Dominic</t>
         </is>
       </c>
       <c r="D790" s="8" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E790" s="8" t="inlineStr">
         <is>
@@ -39466,7 +39466,7 @@
       </c>
       <c r="I790" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Fine Arts</t>
         </is>
       </c>
       <c r="J790" s="8" t="n"/>
@@ -39478,20 +39478,20 @@
     </row>
     <row r="791">
       <c r="A791" s="8" t="n">
-        <v>121196</v>
+        <v>121287</v>
       </c>
       <c r="B791" s="8" t="inlineStr">
         <is>
-          <t>Bocchino</t>
+          <t>Elliott</t>
         </is>
       </c>
       <c r="C791" s="8" t="inlineStr">
         <is>
-          <t>Dominic</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="D791" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E791" s="8" t="inlineStr">
         <is>
@@ -39515,7 +39515,7 @@
       </c>
       <c r="I791" s="8" t="inlineStr">
         <is>
-          <t>Fine Arts</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J791" s="8" t="n"/>
@@ -39527,20 +39527,20 @@
     </row>
     <row r="792">
       <c r="A792" s="8" t="n">
-        <v>121287</v>
+        <v>121290</v>
       </c>
       <c r="B792" s="8" t="inlineStr">
         <is>
-          <t>Elliott</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="C792" s="8" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Jack</t>
         </is>
       </c>
       <c r="D792" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E792" s="8" t="inlineStr">
         <is>
@@ -39564,7 +39564,7 @@
       </c>
       <c r="I792" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J792" s="8" t="n"/>
@@ -39576,11 +39576,11 @@
     </row>
     <row r="793">
       <c r="A793" s="8" t="n">
-        <v>121290</v>
+        <v>121305</v>
       </c>
       <c r="B793" s="8" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Minks</t>
         </is>
       </c>
       <c r="C793" s="8" t="inlineStr">
@@ -39625,20 +39625,20 @@
     </row>
     <row r="794">
       <c r="A794" s="8" t="n">
-        <v>121305</v>
+        <v>121320</v>
       </c>
       <c r="B794" s="8" t="inlineStr">
         <is>
-          <t>Minks</t>
+          <t>Kirby</t>
         </is>
       </c>
       <c r="C794" s="8" t="inlineStr">
         <is>
-          <t>Jack</t>
+          <t>Benjamin</t>
         </is>
       </c>
       <c r="D794" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E794" s="8" t="inlineStr">
         <is>
@@ -39662,7 +39662,7 @@
       </c>
       <c r="I794" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J794" s="8" t="n"/>
@@ -39674,20 +39674,20 @@
     </row>
     <row r="795">
       <c r="A795" s="8" t="n">
-        <v>121320</v>
+        <v>121341</v>
       </c>
       <c r="B795" s="8" t="inlineStr">
         <is>
-          <t>Kirby</t>
+          <t>Jaroszuk</t>
         </is>
       </c>
       <c r="C795" s="8" t="inlineStr">
         <is>
-          <t>Benjamin</t>
+          <t>Nikodem</t>
         </is>
       </c>
       <c r="D795" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E795" s="8" t="inlineStr">
         <is>
@@ -39711,7 +39711,7 @@
       </c>
       <c r="I795" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J795" s="8" t="n"/>
@@ -39723,20 +39723,20 @@
     </row>
     <row r="796">
       <c r="A796" s="8" t="n">
-        <v>121341</v>
+        <v>121384</v>
       </c>
       <c r="B796" s="8" t="inlineStr">
         <is>
-          <t>Jaroszuk</t>
+          <t>Ryzy</t>
         </is>
       </c>
       <c r="C796" s="8" t="inlineStr">
         <is>
-          <t>Nikodem</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="D796" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E796" s="8" t="inlineStr">
         <is>
@@ -39760,7 +39760,7 @@
       </c>
       <c r="I796" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J796" s="8" t="n"/>
@@ -39772,20 +39772,20 @@
     </row>
     <row r="797">
       <c r="A797" s="8" t="n">
-        <v>121384</v>
+        <v>121423</v>
       </c>
       <c r="B797" s="8" t="inlineStr">
         <is>
-          <t>Ryzy</t>
+          <t>Darin</t>
         </is>
       </c>
       <c r="C797" s="8" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="D797" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E797" s="8" t="inlineStr">
         <is>
@@ -39809,7 +39809,7 @@
       </c>
       <c r="I797" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Communication Arts</t>
         </is>
       </c>
       <c r="J797" s="8" t="n"/>
@@ -39821,20 +39821,20 @@
     </row>
     <row r="798">
       <c r="A798" s="8" t="n">
-        <v>121423</v>
+        <v>121441</v>
       </c>
       <c r="B798" s="8" t="inlineStr">
         <is>
-          <t>Darin</t>
+          <t>Wyda</t>
         </is>
       </c>
       <c r="C798" s="8" t="inlineStr">
         <is>
-          <t>Max</t>
+          <t>Andrew</t>
         </is>
       </c>
       <c r="D798" s="8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E798" s="8" t="inlineStr">
         <is>
@@ -39858,7 +39858,7 @@
       </c>
       <c r="I798" s="8" t="inlineStr">
         <is>
-          <t>Communication Arts</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J798" s="8" t="n"/>
@@ -39870,20 +39870,20 @@
     </row>
     <row r="799">
       <c r="A799" s="8" t="n">
-        <v>121441</v>
+        <v>121444</v>
       </c>
       <c r="B799" s="8" t="inlineStr">
         <is>
-          <t>Wyda</t>
+          <t>Diamantis</t>
         </is>
       </c>
       <c r="C799" s="8" t="inlineStr">
         <is>
-          <t>Andrew</t>
+          <t>Oliver</t>
         </is>
       </c>
       <c r="D799" s="8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E799" s="8" t="inlineStr">
         <is>
@@ -39907,7 +39907,7 @@
       </c>
       <c r="I799" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Theater</t>
         </is>
       </c>
       <c r="J799" s="8" t="n"/>
@@ -39919,20 +39919,20 @@
     </row>
     <row r="800">
       <c r="A800" s="8" t="n">
-        <v>121444</v>
+        <v>121491</v>
       </c>
       <c r="B800" s="8" t="inlineStr">
         <is>
-          <t>Diamantis</t>
+          <t>Trotman</t>
         </is>
       </c>
       <c r="C800" s="8" t="inlineStr">
         <is>
-          <t>Oliver</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="D800" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E800" s="8" t="inlineStr">
         <is>
@@ -39956,7 +39956,7 @@
       </c>
       <c r="I800" s="8" t="inlineStr">
         <is>
-          <t>Theater</t>
+          <t>Fine Arts</t>
         </is>
       </c>
       <c r="J800" s="8" t="n"/>
@@ -39968,16 +39968,16 @@
     </row>
     <row r="801">
       <c r="A801" s="8" t="n">
-        <v>121491</v>
+        <v>121758</v>
       </c>
       <c r="B801" s="8" t="inlineStr">
         <is>
-          <t>Trotman</t>
+          <t>Iacono</t>
         </is>
       </c>
       <c r="C801" s="8" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Dylan</t>
         </is>
       </c>
       <c r="D801" s="8" t="n">
@@ -40005,7 +40005,7 @@
       </c>
       <c r="I801" s="8" t="inlineStr">
         <is>
-          <t>Fine Arts</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J801" s="8" t="n"/>
@@ -40017,16 +40017,16 @@
     </row>
     <row r="802">
       <c r="A802" s="8" t="n">
-        <v>121758</v>
+        <v>121826</v>
       </c>
       <c r="B802" s="8" t="inlineStr">
         <is>
-          <t>Iacono</t>
+          <t>Slominsky</t>
         </is>
       </c>
       <c r="C802" s="8" t="inlineStr">
         <is>
-          <t>Dylan</t>
+          <t>Antonio</t>
         </is>
       </c>
       <c r="D802" s="8" t="n">
@@ -40054,7 +40054,7 @@
       </c>
       <c r="I802" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="J802" s="8" t="n"/>
@@ -40066,20 +40066,20 @@
     </row>
     <row r="803">
       <c r="A803" s="8" t="n">
-        <v>121826</v>
+        <v>121842</v>
       </c>
       <c r="B803" s="8" t="inlineStr">
         <is>
-          <t>Slominsky</t>
+          <t>Ritcher</t>
         </is>
       </c>
       <c r="C803" s="8" t="inlineStr">
         <is>
-          <t>Antonio</t>
+          <t>William</t>
         </is>
       </c>
       <c r="D803" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E803" s="8" t="inlineStr">
         <is>
@@ -40103,7 +40103,7 @@
       </c>
       <c r="I803" s="8" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Music Arts</t>
         </is>
       </c>
       <c r="J803" s="8" t="n"/>
@@ -40115,20 +40115,20 @@
     </row>
     <row r="804">
       <c r="A804" s="8" t="n">
-        <v>121842</v>
+        <v>121949</v>
       </c>
       <c r="B804" s="8" t="inlineStr">
         <is>
-          <t>Ritcher</t>
+          <t>Ferko</t>
         </is>
       </c>
       <c r="C804" s="8" t="inlineStr">
         <is>
-          <t>William</t>
+          <t>Lavdosh</t>
         </is>
       </c>
       <c r="D804" s="8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E804" s="8" t="inlineStr">
         <is>
@@ -40152,7 +40152,7 @@
       </c>
       <c r="I804" s="8" t="inlineStr">
         <is>
-          <t>Music Arts</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J804" s="8" t="n"/>
@@ -40164,16 +40164,16 @@
     </row>
     <row r="805">
       <c r="A805" s="8" t="n">
-        <v>121949</v>
+        <v>121986</v>
       </c>
       <c r="B805" s="8" t="inlineStr">
         <is>
-          <t>Ferko</t>
+          <t>Rodriguez</t>
         </is>
       </c>
       <c r="C805" s="8" t="inlineStr">
         <is>
-          <t>Lavdosh</t>
+          <t>Blake</t>
         </is>
       </c>
       <c r="D805" s="8" t="n">
@@ -40212,98 +40212,49 @@
       </c>
     </row>
     <row r="806">
-      <c r="A806" s="8" t="n">
-        <v>121986</v>
-      </c>
-      <c r="B806" s="8" t="inlineStr">
-        <is>
-          <t>Rodriguez</t>
-        </is>
-      </c>
-      <c r="C806" s="8" t="inlineStr">
-        <is>
-          <t>Blake</t>
-        </is>
-      </c>
-      <c r="D806" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="E806" s="8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F806" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G806" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H806" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I806" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J806" s="8" t="n"/>
-      <c r="K806" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="807">
-      <c r="A807" s="15" t="n">
+      <c r="A806" s="15" t="n">
         <v>122015</v>
       </c>
-      <c r="B807" s="15" t="inlineStr">
+      <c r="B806" s="15" t="inlineStr">
         <is>
           <t>Vega</t>
         </is>
       </c>
-      <c r="C807" s="15" t="inlineStr">
+      <c r="C806" s="15" t="inlineStr">
         <is>
           <t>Matthew</t>
         </is>
       </c>
-      <c r="D807" s="7" t="n">
+      <c r="D806" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="E807" s="15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F807" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G807" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H807" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I807" s="15" t="inlineStr">
+      <c r="E806" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F806" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G806" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H806" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I806" s="15" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="J807" s="18" t="n"/>
-      <c r="K807" s="18" t="inlineStr">
+      <c r="J806" s="18" t="n"/>
+      <c r="K806" s="18" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>